<commit_message>
Added readme files for every relevant folder except "verification" folder (will be done seperately, only due to time management). Solved Supplementary materials issue (seperate numbering and correct cross-referencing) and moved 3 supp figures to the last section. Rendered index.
</commit_message>
<xml_diff>
--- a/main_folders_structure.xlsx
+++ b/main_folders_structure.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AVIHAY\git\DCC-v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94C184C5-1F25-4A5E-96F4-2F2D92E4ADD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737DA663-2A00-4A1D-BC58-017C505A2672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19080" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9331410C-6D9F-4602-9E3C-4D4BE81F6669}"/>
   </bookViews>
@@ -243,7 +243,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -256,8 +256,20 @@
       <name val="Fira Code"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Trebuchet MS"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1" tint="0.499984740745262"/>
+      <name val="Fira Code"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,6 +279,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -283,12 +301,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,89 +649,90 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{534B8491-E878-427A-A9B9-32F7AB888376}">
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:B76"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B2" s="4"/>
+    </row>
+    <row r="3" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:2" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -849,118 +876,118 @@
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
+    <row r="45" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
+    <row r="47" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A48" s="1" t="s">
+    <row r="48" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A49" s="1" t="s">
+    <row r="49" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A51" s="1" t="s">
+    <row r="51" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A52" s="1" t="s">
+    <row r="52" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A53" s="1" t="s">
+    <row r="53" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A54" s="1" t="s">
+    <row r="54" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A55" s="1" t="s">
+    <row r="55" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
+    <row r="58" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
+    <row r="59" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
+    <row r="60" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="6" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
+    <row r="61" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A63" s="1" t="s">
+    <row r="63" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A64" s="1" t="s">
+    <row r="64" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A65" s="1" t="s">
+    <row r="65" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A66" s="1" t="s">
+    <row r="66" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A67" s="1" t="s">
+    <row r="67" spans="1:1" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
         <v>65</v>
       </c>
     </row>
@@ -993,5 +1020,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>